<commit_message>
Finalizado el luchador y otras clases
</commit_message>
<xml_diff>
--- a/Excels compiladores de habilidades/Habilidades de criaturas no humanoides.xlsx
+++ b/Excels compiladores de habilidades/Habilidades de criaturas no humanoides.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Lenovo\arkanor-assets\Excels compiladores de habilidades\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F3E19B80-8EF5-4008-874F-A7259BC75378}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{203E564D-1191-400D-A04A-3554C52244FE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" xr2:uid="{4E5D0542-3908-4101-9CFE-772E035496F2}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" activeTab="4" xr2:uid="{4E5D0542-3908-4101-9CFE-772E035496F2}"/>
   </bookViews>
   <sheets>
     <sheet name="No-Muerto" sheetId="8" r:id="rId1"/>
@@ -9494,15 +9494,6 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="10" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="10" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -9516,6 +9507,15 @@
     </xf>
     <xf numFmtId="0" fontId="9" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -12439,15 +12439,15 @@
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
       <xdr:col>9</xdr:col>
-      <xdr:colOff>47224</xdr:colOff>
-      <xdr:row>0</xdr:row>
-      <xdr:rowOff>346900</xdr:rowOff>
+      <xdr:colOff>36019</xdr:colOff>
+      <xdr:row>1</xdr:row>
+      <xdr:rowOff>10723</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>9</xdr:col>
-      <xdr:colOff>735267</xdr:colOff>
-      <xdr:row>2</xdr:row>
-      <xdr:rowOff>340178</xdr:rowOff>
+      <xdr:colOff>724062</xdr:colOff>
+      <xdr:row>3</xdr:row>
+      <xdr:rowOff>4001</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -12476,8 +12476,8 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="6905224" y="346900"/>
-          <a:ext cx="688043" cy="700849"/>
+          <a:off x="6894019" y="358105"/>
+          <a:ext cx="688043" cy="688043"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -12639,13 +12639,13 @@
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
       <xdr:col>7</xdr:col>
-      <xdr:colOff>27214</xdr:colOff>
+      <xdr:colOff>49626</xdr:colOff>
       <xdr:row>10</xdr:row>
       <xdr:rowOff>13607</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>7</xdr:col>
-      <xdr:colOff>711214</xdr:colOff>
+      <xdr:colOff>733626</xdr:colOff>
       <xdr:row>11</xdr:row>
       <xdr:rowOff>343821</xdr:rowOff>
     </xdr:to>
@@ -12676,8 +12676,8 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="5361214" y="3551464"/>
-          <a:ext cx="684000" cy="684000"/>
+          <a:off x="5383626" y="3487431"/>
+          <a:ext cx="684000" cy="677596"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -15333,7 +15333,7 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:18" ht="27.95" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="17"/>
+      <c r="A1" s="22"/>
       <c r="B1" s="14"/>
       <c r="C1" s="7"/>
       <c r="D1" s="7"/>
@@ -15349,7 +15349,7 @@
       <c r="N1" s="7"/>
     </row>
     <row r="2" spans="1:18" ht="27.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="18"/>
+      <c r="A2" s="23"/>
       <c r="B2" s="15"/>
       <c r="C2" s="15"/>
       <c r="D2" s="15"/>
@@ -15365,7 +15365,7 @@
       <c r="N2" s="15"/>
     </row>
     <row r="3" spans="1:18" ht="27.95" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="19"/>
+      <c r="A3" s="24"/>
       <c r="B3" s="16"/>
       <c r="C3" s="16"/>
       <c r="D3" s="16"/>
@@ -15381,7 +15381,7 @@
       <c r="N3" s="16"/>
     </row>
     <row r="4" spans="1:18" ht="27.95" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A4" s="20"/>
+      <c r="A4" s="17"/>
       <c r="B4" s="14"/>
       <c r="C4" s="7"/>
       <c r="D4" s="7"/>
@@ -15397,7 +15397,7 @@
       <c r="N4" s="7"/>
     </row>
     <row r="5" spans="1:18" ht="27.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="21"/>
+      <c r="A5" s="18"/>
       <c r="B5" s="15"/>
       <c r="C5" s="15"/>
       <c r="D5" s="15"/>
@@ -15413,7 +15413,7 @@
       <c r="N5" s="15"/>
     </row>
     <row r="6" spans="1:18" ht="27.95" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A6" s="22"/>
+      <c r="A6" s="19"/>
       <c r="B6" s="16"/>
       <c r="C6" s="16"/>
       <c r="D6" s="16"/>
@@ -15429,7 +15429,7 @@
       <c r="N6" s="16"/>
     </row>
     <row r="7" spans="1:18" ht="27.95" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A7" s="20"/>
+      <c r="A7" s="17"/>
       <c r="B7" s="7"/>
       <c r="C7" s="7"/>
       <c r="D7" s="7"/>
@@ -15445,12 +15445,12 @@
       <c r="N7" s="7"/>
     </row>
     <row r="8" spans="1:18" ht="27.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A8" s="21"/>
+      <c r="A8" s="18"/>
       <c r="B8" s="15"/>
       <c r="C8" s="15"/>
       <c r="D8" s="15"/>
       <c r="E8" s="15"/>
-      <c r="F8" s="23"/>
+      <c r="F8" s="20"/>
       <c r="G8" s="15"/>
       <c r="H8" s="15"/>
       <c r="I8" s="15"/>
@@ -15461,12 +15461,12 @@
       <c r="N8" s="15"/>
     </row>
     <row r="9" spans="1:18" ht="27.95" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A9" s="22"/>
+      <c r="A9" s="19"/>
       <c r="B9" s="16"/>
       <c r="C9" s="16"/>
       <c r="D9" s="16"/>
       <c r="E9" s="16"/>
-      <c r="F9" s="24"/>
+      <c r="F9" s="21"/>
       <c r="G9" s="16"/>
       <c r="H9" s="16"/>
       <c r="I9" s="16"/>
@@ -15478,7 +15478,7 @@
       <c r="R9" s="10"/>
     </row>
     <row r="10" spans="1:18" ht="27.95" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A10" s="20"/>
+      <c r="A10" s="17"/>
       <c r="B10" s="7"/>
       <c r="C10" s="7"/>
       <c r="D10" s="7"/>
@@ -15494,7 +15494,7 @@
       <c r="N10" s="7"/>
     </row>
     <row r="11" spans="1:18" ht="27.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A11" s="21"/>
+      <c r="A11" s="18"/>
       <c r="B11" s="15"/>
       <c r="C11" s="15"/>
       <c r="D11" s="15"/>
@@ -15510,7 +15510,7 @@
       <c r="N11" s="15"/>
     </row>
     <row r="12" spans="1:18" ht="27.95" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A12" s="22"/>
+      <c r="A12" s="19"/>
       <c r="B12" s="16"/>
       <c r="C12" s="16"/>
       <c r="D12" s="16"/>
@@ -15526,7 +15526,7 @@
       <c r="N12" s="16"/>
     </row>
     <row r="13" spans="1:18" ht="27.95" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A13" s="20"/>
+      <c r="A13" s="17"/>
       <c r="B13" s="7"/>
       <c r="C13" s="7"/>
       <c r="D13" s="9"/>
@@ -15542,7 +15542,7 @@
       <c r="N13" s="7"/>
     </row>
     <row r="14" spans="1:18" ht="27.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A14" s="21"/>
+      <c r="A14" s="18"/>
       <c r="B14" s="15"/>
       <c r="C14" s="15"/>
       <c r="D14" s="15"/>
@@ -15558,7 +15558,342 @@
       <c r="N14" s="15"/>
     </row>
     <row r="15" spans="1:18" ht="27.95" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A15" s="22"/>
+      <c r="A15" s="19"/>
+      <c r="B15" s="16"/>
+      <c r="C15" s="16"/>
+      <c r="D15" s="16"/>
+      <c r="E15" s="16"/>
+      <c r="F15" s="16"/>
+      <c r="G15" s="16"/>
+      <c r="H15" s="16"/>
+      <c r="I15" s="16"/>
+      <c r="J15" s="16"/>
+      <c r="K15" s="16"/>
+      <c r="L15" s="16"/>
+      <c r="M15" s="16"/>
+      <c r="N15" s="16"/>
+    </row>
+  </sheetData>
+  <mergeCells count="70">
+    <mergeCell ref="L2:L3"/>
+    <mergeCell ref="A1:A3"/>
+    <mergeCell ref="B2:B3"/>
+    <mergeCell ref="C2:C3"/>
+    <mergeCell ref="D2:D3"/>
+    <mergeCell ref="E2:E3"/>
+    <mergeCell ref="F2:F3"/>
+    <mergeCell ref="N5:N6"/>
+    <mergeCell ref="M2:M3"/>
+    <mergeCell ref="N2:N3"/>
+    <mergeCell ref="A4:A6"/>
+    <mergeCell ref="B5:B6"/>
+    <mergeCell ref="C5:C6"/>
+    <mergeCell ref="D5:D6"/>
+    <mergeCell ref="E5:E6"/>
+    <mergeCell ref="F5:F6"/>
+    <mergeCell ref="G5:G6"/>
+    <mergeCell ref="H5:H6"/>
+    <mergeCell ref="G2:G3"/>
+    <mergeCell ref="H2:H3"/>
+    <mergeCell ref="I2:I3"/>
+    <mergeCell ref="J2:J3"/>
+    <mergeCell ref="K2:K3"/>
+    <mergeCell ref="I5:I6"/>
+    <mergeCell ref="J5:J6"/>
+    <mergeCell ref="K5:K6"/>
+    <mergeCell ref="L5:L6"/>
+    <mergeCell ref="M5:M6"/>
+    <mergeCell ref="K8:K9"/>
+    <mergeCell ref="L8:L9"/>
+    <mergeCell ref="A7:A9"/>
+    <mergeCell ref="B8:B9"/>
+    <mergeCell ref="C8:C9"/>
+    <mergeCell ref="D8:D9"/>
+    <mergeCell ref="E8:E9"/>
+    <mergeCell ref="F8:F9"/>
+    <mergeCell ref="M11:M12"/>
+    <mergeCell ref="N11:N12"/>
+    <mergeCell ref="M8:M9"/>
+    <mergeCell ref="N8:N9"/>
+    <mergeCell ref="A10:A12"/>
+    <mergeCell ref="B11:B12"/>
+    <mergeCell ref="C11:C12"/>
+    <mergeCell ref="D11:D12"/>
+    <mergeCell ref="E11:E12"/>
+    <mergeCell ref="F11:F12"/>
+    <mergeCell ref="G11:G12"/>
+    <mergeCell ref="H11:H12"/>
+    <mergeCell ref="G8:G9"/>
+    <mergeCell ref="H8:H9"/>
+    <mergeCell ref="I8:I9"/>
+    <mergeCell ref="J8:J9"/>
+    <mergeCell ref="F14:F15"/>
+    <mergeCell ref="I11:I12"/>
+    <mergeCell ref="J11:J12"/>
+    <mergeCell ref="K11:K12"/>
+    <mergeCell ref="L11:L12"/>
+    <mergeCell ref="A13:A15"/>
+    <mergeCell ref="B14:B15"/>
+    <mergeCell ref="C14:C15"/>
+    <mergeCell ref="D14:D15"/>
+    <mergeCell ref="E14:E15"/>
+    <mergeCell ref="M14:M15"/>
+    <mergeCell ref="N14:N15"/>
+    <mergeCell ref="G14:G15"/>
+    <mergeCell ref="H14:H15"/>
+    <mergeCell ref="I14:I15"/>
+    <mergeCell ref="J14:J15"/>
+    <mergeCell ref="K14:K15"/>
+    <mergeCell ref="L14:L15"/>
+  </mergeCells>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <legacyDrawing r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8D5F5BAF-BE93-4F06-A7C2-0B0CBE1C14C1}">
+  <dimension ref="A1:R15"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="27.95" customHeight="1" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="16384" width="11.42578125" style="6"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:18" ht="27.95" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A1" s="22" t="s">
+        <v>116</v>
+      </c>
+      <c r="B1" s="14" t="s">
+        <v>115</v>
+      </c>
+      <c r="C1" s="7" t="s">
+        <v>118</v>
+      </c>
+      <c r="D1" s="7" t="s">
+        <v>117</v>
+      </c>
+      <c r="E1" s="7"/>
+      <c r="F1" s="7"/>
+      <c r="G1" s="7"/>
+      <c r="H1" s="7"/>
+      <c r="I1" s="7"/>
+      <c r="J1" s="7"/>
+      <c r="K1" s="7"/>
+      <c r="L1" s="7"/>
+      <c r="M1" s="7"/>
+      <c r="N1" s="7"/>
+    </row>
+    <row r="2" spans="1:18" ht="27.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A2" s="23"/>
+      <c r="B2" s="15"/>
+      <c r="C2" s="15"/>
+      <c r="D2" s="15"/>
+      <c r="E2" s="15"/>
+      <c r="F2" s="15"/>
+      <c r="G2" s="15"/>
+      <c r="H2" s="15"/>
+      <c r="I2" s="15"/>
+      <c r="J2" s="15"/>
+      <c r="K2" s="15"/>
+      <c r="L2" s="15"/>
+      <c r="M2" s="15"/>
+      <c r="N2" s="15"/>
+    </row>
+    <row r="3" spans="1:18" ht="27.95" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A3" s="24"/>
+      <c r="B3" s="16"/>
+      <c r="C3" s="16"/>
+      <c r="D3" s="16"/>
+      <c r="E3" s="16"/>
+      <c r="F3" s="16"/>
+      <c r="G3" s="16"/>
+      <c r="H3" s="16"/>
+      <c r="I3" s="16"/>
+      <c r="J3" s="16"/>
+      <c r="K3" s="16"/>
+      <c r="L3" s="16"/>
+      <c r="M3" s="16"/>
+      <c r="N3" s="16"/>
+    </row>
+    <row r="4" spans="1:18" ht="27.95" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A4" s="17"/>
+      <c r="B4" s="14"/>
+      <c r="C4" s="7"/>
+      <c r="D4" s="7"/>
+      <c r="E4" s="7"/>
+      <c r="F4" s="7"/>
+      <c r="G4" s="7"/>
+      <c r="H4" s="7"/>
+      <c r="I4" s="7"/>
+      <c r="J4" s="7"/>
+      <c r="K4" s="7"/>
+      <c r="L4" s="7"/>
+      <c r="M4" s="7"/>
+      <c r="N4" s="7"/>
+    </row>
+    <row r="5" spans="1:18" ht="27.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A5" s="18"/>
+      <c r="B5" s="15"/>
+      <c r="C5" s="15"/>
+      <c r="D5" s="15"/>
+      <c r="E5" s="15"/>
+      <c r="F5" s="15"/>
+      <c r="G5" s="15"/>
+      <c r="H5" s="15"/>
+      <c r="I5" s="15"/>
+      <c r="J5" s="15"/>
+      <c r="K5" s="15"/>
+      <c r="L5" s="15"/>
+      <c r="M5" s="15"/>
+      <c r="N5" s="15"/>
+    </row>
+    <row r="6" spans="1:18" ht="27.95" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A6" s="19"/>
+      <c r="B6" s="16"/>
+      <c r="C6" s="16"/>
+      <c r="D6" s="16"/>
+      <c r="E6" s="16"/>
+      <c r="F6" s="16"/>
+      <c r="G6" s="16"/>
+      <c r="H6" s="16"/>
+      <c r="I6" s="16"/>
+      <c r="J6" s="16"/>
+      <c r="K6" s="16"/>
+      <c r="L6" s="16"/>
+      <c r="M6" s="16"/>
+      <c r="N6" s="16"/>
+    </row>
+    <row r="7" spans="1:18" ht="27.95" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A7" s="17"/>
+      <c r="B7" s="7"/>
+      <c r="C7" s="7"/>
+      <c r="D7" s="7"/>
+      <c r="E7" s="7"/>
+      <c r="F7" s="9"/>
+      <c r="G7" s="7"/>
+      <c r="H7" s="7"/>
+      <c r="I7" s="7"/>
+      <c r="J7" s="7"/>
+      <c r="K7" s="7"/>
+      <c r="L7" s="7"/>
+      <c r="M7" s="7"/>
+      <c r="N7" s="7"/>
+    </row>
+    <row r="8" spans="1:18" ht="27.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A8" s="18"/>
+      <c r="B8" s="15"/>
+      <c r="C8" s="15"/>
+      <c r="D8" s="15"/>
+      <c r="E8" s="15"/>
+      <c r="F8" s="20"/>
+      <c r="G8" s="15"/>
+      <c r="H8" s="15"/>
+      <c r="I8" s="15"/>
+      <c r="J8" s="15"/>
+      <c r="K8" s="15"/>
+      <c r="L8" s="15"/>
+      <c r="M8" s="15"/>
+      <c r="N8" s="15"/>
+    </row>
+    <row r="9" spans="1:18" ht="27.95" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A9" s="19"/>
+      <c r="B9" s="16"/>
+      <c r="C9" s="16"/>
+      <c r="D9" s="16"/>
+      <c r="E9" s="16"/>
+      <c r="F9" s="21"/>
+      <c r="G9" s="16"/>
+      <c r="H9" s="16"/>
+      <c r="I9" s="16"/>
+      <c r="J9" s="16"/>
+      <c r="K9" s="16"/>
+      <c r="L9" s="16"/>
+      <c r="M9" s="16"/>
+      <c r="N9" s="16"/>
+      <c r="R9" s="10"/>
+    </row>
+    <row r="10" spans="1:18" ht="27.95" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A10" s="17"/>
+      <c r="B10" s="7"/>
+      <c r="C10" s="7"/>
+      <c r="D10" s="7"/>
+      <c r="E10" s="8"/>
+      <c r="F10" s="7"/>
+      <c r="G10" s="7"/>
+      <c r="H10" s="7"/>
+      <c r="I10" s="7"/>
+      <c r="J10" s="7"/>
+      <c r="K10" s="7"/>
+      <c r="L10" s="7"/>
+      <c r="M10" s="7"/>
+      <c r="N10" s="7"/>
+    </row>
+    <row r="11" spans="1:18" ht="27.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A11" s="18"/>
+      <c r="B11" s="15"/>
+      <c r="C11" s="15"/>
+      <c r="D11" s="15"/>
+      <c r="E11" s="15"/>
+      <c r="F11" s="15"/>
+      <c r="G11" s="15"/>
+      <c r="H11" s="15"/>
+      <c r="I11" s="15"/>
+      <c r="J11" s="15"/>
+      <c r="K11" s="15"/>
+      <c r="L11" s="15"/>
+      <c r="M11" s="15"/>
+      <c r="N11" s="15"/>
+    </row>
+    <row r="12" spans="1:18" ht="27.95" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A12" s="19"/>
+      <c r="B12" s="16"/>
+      <c r="C12" s="16"/>
+      <c r="D12" s="16"/>
+      <c r="E12" s="16"/>
+      <c r="F12" s="16"/>
+      <c r="G12" s="16"/>
+      <c r="H12" s="16"/>
+      <c r="I12" s="16"/>
+      <c r="J12" s="16"/>
+      <c r="K12" s="16"/>
+      <c r="L12" s="16"/>
+      <c r="M12" s="16"/>
+      <c r="N12" s="16"/>
+    </row>
+    <row r="13" spans="1:18" ht="27.95" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A13" s="17"/>
+      <c r="B13" s="7"/>
+      <c r="C13" s="7"/>
+      <c r="D13" s="9"/>
+      <c r="E13" s="7"/>
+      <c r="F13" s="7"/>
+      <c r="G13" s="7"/>
+      <c r="H13" s="7"/>
+      <c r="I13" s="7"/>
+      <c r="J13" s="7"/>
+      <c r="K13" s="7"/>
+      <c r="L13" s="9"/>
+      <c r="M13" s="7"/>
+      <c r="N13" s="7"/>
+    </row>
+    <row r="14" spans="1:18" ht="27.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A14" s="18"/>
+      <c r="B14" s="15"/>
+      <c r="C14" s="15"/>
+      <c r="D14" s="15"/>
+      <c r="E14" s="15"/>
+      <c r="F14" s="15"/>
+      <c r="G14" s="15"/>
+      <c r="H14" s="15"/>
+      <c r="I14" s="15"/>
+      <c r="J14" s="15"/>
+      <c r="K14" s="15"/>
+      <c r="L14" s="15"/>
+      <c r="M14" s="15"/>
+      <c r="N14" s="15"/>
+    </row>
+    <row r="15" spans="1:18" ht="27.95" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A15" s="19"/>
       <c r="B15" s="16"/>
       <c r="C15" s="16"/>
       <c r="D15" s="16"/>
@@ -15647,12 +15982,13 @@
     <mergeCell ref="F2:F3"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <legacyDrawing r:id="rId1"/>
+  <drawing r:id="rId1"/>
+  <legacyDrawing r:id="rId2"/>
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8D5F5BAF-BE93-4F06-A7C2-0B0CBE1C14C1}">
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A9F6337B-89AA-4305-B4A8-6D5D44FBF989}">
   <dimension ref="A1:R15"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="27.95" customHeight="1" x14ac:dyDescent="0.25"/>
   <cols>
@@ -15660,18 +15996,14 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:18" ht="27.95" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="17" t="s">
-        <v>116</v>
-      </c>
+      <c r="A1" s="22"/>
       <c r="B1" s="14" t="s">
-        <v>115</v>
+        <v>103</v>
       </c>
       <c r="C1" s="7" t="s">
-        <v>118</v>
+        <v>122</v>
       </c>
-      <c r="D1" s="7" t="s">
-        <v>117</v>
-      </c>
+      <c r="D1" s="7"/>
       <c r="E1" s="7"/>
       <c r="F1" s="7"/>
       <c r="G1" s="7"/>
@@ -15684,7 +16016,7 @@
       <c r="N1" s="7"/>
     </row>
     <row r="2" spans="1:18" ht="27.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="18"/>
+      <c r="A2" s="23"/>
       <c r="B2" s="15"/>
       <c r="C2" s="15"/>
       <c r="D2" s="15"/>
@@ -15700,7 +16032,7 @@
       <c r="N2" s="15"/>
     </row>
     <row r="3" spans="1:18" ht="27.95" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="19"/>
+      <c r="A3" s="24"/>
       <c r="B3" s="16"/>
       <c r="C3" s="16"/>
       <c r="D3" s="16"/>
@@ -15716,9 +16048,13 @@
       <c r="N3" s="16"/>
     </row>
     <row r="4" spans="1:18" ht="27.95" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A4" s="20"/>
-      <c r="B4" s="14"/>
-      <c r="C4" s="7"/>
+      <c r="A4" s="17"/>
+      <c r="B4" s="14" t="s">
+        <v>104</v>
+      </c>
+      <c r="C4" s="7" t="s">
+        <v>109</v>
+      </c>
       <c r="D4" s="7"/>
       <c r="E4" s="7"/>
       <c r="F4" s="7"/>
@@ -15732,7 +16068,7 @@
       <c r="N4" s="7"/>
     </row>
     <row r="5" spans="1:18" ht="27.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="21"/>
+      <c r="A5" s="18"/>
       <c r="B5" s="15"/>
       <c r="C5" s="15"/>
       <c r="D5" s="15"/>
@@ -15748,7 +16084,7 @@
       <c r="N5" s="15"/>
     </row>
     <row r="6" spans="1:18" ht="27.95" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A6" s="22"/>
+      <c r="A6" s="19"/>
       <c r="B6" s="16"/>
       <c r="C6" s="16"/>
       <c r="D6" s="16"/>
@@ -15764,7 +16100,355 @@
       <c r="N6" s="16"/>
     </row>
     <row r="7" spans="1:18" ht="27.95" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A7" s="20"/>
+      <c r="A7" s="17" t="s">
+        <v>111</v>
+      </c>
+      <c r="B7" s="7" t="s">
+        <v>105</v>
+      </c>
+      <c r="C7" s="7" t="s">
+        <v>106</v>
+      </c>
+      <c r="D7" s="7" t="s">
+        <v>108</v>
+      </c>
+      <c r="E7" s="7" t="s">
+        <v>110</v>
+      </c>
+      <c r="F7" s="7" t="s">
+        <v>121</v>
+      </c>
+      <c r="G7" s="7"/>
+      <c r="H7" s="7"/>
+      <c r="I7" s="7"/>
+      <c r="J7" s="7"/>
+      <c r="K7" s="7"/>
+      <c r="L7" s="7"/>
+      <c r="M7" s="7"/>
+      <c r="N7" s="7"/>
+    </row>
+    <row r="8" spans="1:18" ht="27.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A8" s="18"/>
+      <c r="B8" s="15"/>
+      <c r="C8" s="15"/>
+      <c r="D8" s="15"/>
+      <c r="E8" s="15"/>
+      <c r="F8" s="15"/>
+      <c r="G8" s="15"/>
+      <c r="H8" s="15"/>
+      <c r="I8" s="15"/>
+      <c r="J8" s="15"/>
+      <c r="K8" s="15"/>
+      <c r="L8" s="15"/>
+      <c r="M8" s="15"/>
+      <c r="N8" s="15"/>
+    </row>
+    <row r="9" spans="1:18" ht="27.95" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A9" s="19"/>
+      <c r="B9" s="16"/>
+      <c r="C9" s="16"/>
+      <c r="D9" s="16"/>
+      <c r="E9" s="16"/>
+      <c r="F9" s="16"/>
+      <c r="G9" s="16"/>
+      <c r="H9" s="16"/>
+      <c r="I9" s="16"/>
+      <c r="J9" s="16"/>
+      <c r="K9" s="16"/>
+      <c r="L9" s="16"/>
+      <c r="M9" s="16"/>
+      <c r="N9" s="16"/>
+      <c r="R9" s="10"/>
+    </row>
+    <row r="10" spans="1:18" ht="27.95" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A10" s="17"/>
+      <c r="B10" s="7" t="s">
+        <v>107</v>
+      </c>
+      <c r="C10" s="7" t="s">
+        <v>112</v>
+      </c>
+      <c r="D10" s="7" t="s">
+        <v>113</v>
+      </c>
+      <c r="E10" s="7" t="s">
+        <v>114</v>
+      </c>
+      <c r="F10" s="7"/>
+      <c r="G10" s="7"/>
+      <c r="H10" s="7"/>
+      <c r="I10" s="7"/>
+      <c r="J10" s="7"/>
+      <c r="K10" s="7"/>
+      <c r="L10" s="7"/>
+      <c r="M10" s="7"/>
+      <c r="N10" s="7"/>
+    </row>
+    <row r="11" spans="1:18" ht="27.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A11" s="18"/>
+      <c r="B11" s="15"/>
+      <c r="C11" s="15"/>
+      <c r="D11" s="15"/>
+      <c r="E11" s="15"/>
+      <c r="F11" s="15"/>
+      <c r="G11" s="15"/>
+      <c r="H11" s="15"/>
+      <c r="I11" s="15"/>
+      <c r="J11" s="15"/>
+      <c r="K11" s="15"/>
+      <c r="L11" s="15"/>
+      <c r="M11" s="15"/>
+      <c r="N11" s="15"/>
+    </row>
+    <row r="12" spans="1:18" ht="27.95" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A12" s="19"/>
+      <c r="B12" s="16"/>
+      <c r="C12" s="16"/>
+      <c r="D12" s="16"/>
+      <c r="E12" s="16"/>
+      <c r="F12" s="16"/>
+      <c r="G12" s="16"/>
+      <c r="H12" s="16"/>
+      <c r="I12" s="16"/>
+      <c r="J12" s="16"/>
+      <c r="K12" s="16"/>
+      <c r="L12" s="16"/>
+      <c r="M12" s="16"/>
+      <c r="N12" s="16"/>
+    </row>
+    <row r="13" spans="1:18" ht="27.95" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A13" s="17"/>
+      <c r="B13" s="7"/>
+      <c r="C13" s="7"/>
+      <c r="D13" s="9"/>
+      <c r="E13" s="7"/>
+      <c r="F13" s="7"/>
+      <c r="G13" s="7"/>
+      <c r="H13" s="7"/>
+      <c r="I13" s="7"/>
+      <c r="J13" s="7"/>
+      <c r="K13" s="7"/>
+      <c r="L13" s="9"/>
+      <c r="M13" s="7"/>
+      <c r="N13" s="7"/>
+    </row>
+    <row r="14" spans="1:18" ht="27.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A14" s="18"/>
+      <c r="B14" s="15"/>
+      <c r="C14" s="15"/>
+      <c r="D14" s="15"/>
+      <c r="E14" s="15"/>
+      <c r="F14" s="15"/>
+      <c r="G14" s="15"/>
+      <c r="H14" s="15"/>
+      <c r="I14" s="15"/>
+      <c r="J14" s="15"/>
+      <c r="K14" s="15"/>
+      <c r="L14" s="15"/>
+      <c r="M14" s="15"/>
+      <c r="N14" s="15"/>
+    </row>
+    <row r="15" spans="1:18" ht="27.95" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A15" s="19"/>
+      <c r="B15" s="16"/>
+      <c r="C15" s="16"/>
+      <c r="D15" s="16"/>
+      <c r="E15" s="16"/>
+      <c r="F15" s="16"/>
+      <c r="G15" s="16"/>
+      <c r="H15" s="16"/>
+      <c r="I15" s="16"/>
+      <c r="J15" s="16"/>
+      <c r="K15" s="16"/>
+      <c r="L15" s="16"/>
+      <c r="M15" s="16"/>
+      <c r="N15" s="16"/>
+    </row>
+  </sheetData>
+  <mergeCells count="70">
+    <mergeCell ref="M14:M15"/>
+    <mergeCell ref="N14:N15"/>
+    <mergeCell ref="G14:G15"/>
+    <mergeCell ref="H14:H15"/>
+    <mergeCell ref="I14:I15"/>
+    <mergeCell ref="J14:J15"/>
+    <mergeCell ref="K14:K15"/>
+    <mergeCell ref="L14:L15"/>
+    <mergeCell ref="A13:A15"/>
+    <mergeCell ref="B14:B15"/>
+    <mergeCell ref="C14:C15"/>
+    <mergeCell ref="D14:D15"/>
+    <mergeCell ref="E14:E15"/>
+    <mergeCell ref="F14:F15"/>
+    <mergeCell ref="I11:I12"/>
+    <mergeCell ref="J11:J12"/>
+    <mergeCell ref="K11:K12"/>
+    <mergeCell ref="L11:L12"/>
+    <mergeCell ref="M11:M12"/>
+    <mergeCell ref="N11:N12"/>
+    <mergeCell ref="M8:M9"/>
+    <mergeCell ref="N8:N9"/>
+    <mergeCell ref="A10:A12"/>
+    <mergeCell ref="B11:B12"/>
+    <mergeCell ref="C11:C12"/>
+    <mergeCell ref="D11:D12"/>
+    <mergeCell ref="E11:E12"/>
+    <mergeCell ref="F11:F12"/>
+    <mergeCell ref="G11:G12"/>
+    <mergeCell ref="H11:H12"/>
+    <mergeCell ref="G8:G9"/>
+    <mergeCell ref="H8:H9"/>
+    <mergeCell ref="I8:I9"/>
+    <mergeCell ref="J8:J9"/>
+    <mergeCell ref="K8:K9"/>
+    <mergeCell ref="L8:L9"/>
+    <mergeCell ref="A7:A9"/>
+    <mergeCell ref="B8:B9"/>
+    <mergeCell ref="C8:C9"/>
+    <mergeCell ref="D8:D9"/>
+    <mergeCell ref="E8:E9"/>
+    <mergeCell ref="F8:F9"/>
+    <mergeCell ref="I5:I6"/>
+    <mergeCell ref="J5:J6"/>
+    <mergeCell ref="K5:K6"/>
+    <mergeCell ref="L5:L6"/>
+    <mergeCell ref="M5:M6"/>
+    <mergeCell ref="N5:N6"/>
+    <mergeCell ref="M2:M3"/>
+    <mergeCell ref="N2:N3"/>
+    <mergeCell ref="A4:A6"/>
+    <mergeCell ref="B5:B6"/>
+    <mergeCell ref="C5:C6"/>
+    <mergeCell ref="D5:D6"/>
+    <mergeCell ref="E5:E6"/>
+    <mergeCell ref="F5:F6"/>
+    <mergeCell ref="G5:G6"/>
+    <mergeCell ref="H5:H6"/>
+    <mergeCell ref="G2:G3"/>
+    <mergeCell ref="H2:H3"/>
+    <mergeCell ref="I2:I3"/>
+    <mergeCell ref="J2:J3"/>
+    <mergeCell ref="K2:K3"/>
+    <mergeCell ref="L2:L3"/>
+    <mergeCell ref="A1:A3"/>
+    <mergeCell ref="B2:B3"/>
+    <mergeCell ref="C2:C3"/>
+    <mergeCell ref="D2:D3"/>
+    <mergeCell ref="E2:E3"/>
+    <mergeCell ref="F2:F3"/>
+  </mergeCells>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <drawing r:id="rId1"/>
+  <legacyDrawing r:id="rId2"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{258ECD2D-C047-4967-AAA4-94D91ED5B3F1}">
+  <dimension ref="A1:R15"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="27.95" customHeight="1" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="16384" width="11.42578125" style="6"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:18" ht="27.95" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A1" s="22"/>
+      <c r="B1" s="7"/>
+      <c r="C1" s="7"/>
+      <c r="D1" s="7"/>
+      <c r="E1" s="7"/>
+      <c r="F1" s="7"/>
+      <c r="G1" s="7"/>
+      <c r="H1" s="7"/>
+      <c r="I1" s="7"/>
+      <c r="J1" s="7"/>
+      <c r="K1" s="7"/>
+      <c r="L1" s="7"/>
+      <c r="M1" s="7"/>
+      <c r="N1" s="7"/>
+    </row>
+    <row r="2" spans="1:18" ht="27.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A2" s="23"/>
+      <c r="B2" s="15"/>
+      <c r="C2" s="15"/>
+      <c r="D2" s="15"/>
+      <c r="E2" s="15"/>
+      <c r="F2" s="15"/>
+      <c r="G2" s="15"/>
+      <c r="H2" s="15"/>
+      <c r="I2" s="15"/>
+      <c r="J2" s="15"/>
+      <c r="K2" s="15"/>
+      <c r="L2" s="15"/>
+      <c r="M2" s="15"/>
+      <c r="N2" s="15"/>
+    </row>
+    <row r="3" spans="1:18" ht="27.95" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A3" s="24"/>
+      <c r="B3" s="16"/>
+      <c r="C3" s="16"/>
+      <c r="D3" s="16"/>
+      <c r="E3" s="16"/>
+      <c r="F3" s="16"/>
+      <c r="G3" s="16"/>
+      <c r="H3" s="16"/>
+      <c r="I3" s="16"/>
+      <c r="J3" s="16"/>
+      <c r="K3" s="16"/>
+      <c r="L3" s="16"/>
+      <c r="M3" s="16"/>
+      <c r="N3" s="16"/>
+    </row>
+    <row r="4" spans="1:18" ht="27.95" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A4" s="17"/>
+      <c r="B4" s="7"/>
+      <c r="C4" s="7"/>
+      <c r="D4" s="7"/>
+      <c r="E4" s="7"/>
+      <c r="F4" s="7"/>
+      <c r="G4" s="7"/>
+      <c r="H4" s="7"/>
+      <c r="I4" s="7"/>
+      <c r="J4" s="7"/>
+      <c r="K4" s="7"/>
+      <c r="L4" s="7"/>
+      <c r="M4" s="7"/>
+      <c r="N4" s="7"/>
+    </row>
+    <row r="5" spans="1:18" ht="27.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A5" s="18"/>
+      <c r="B5" s="15"/>
+      <c r="C5" s="15"/>
+      <c r="D5" s="15"/>
+      <c r="E5" s="15"/>
+      <c r="F5" s="15"/>
+      <c r="G5" s="15"/>
+      <c r="H5" s="15"/>
+      <c r="I5" s="15"/>
+      <c r="J5" s="15"/>
+      <c r="K5" s="15"/>
+      <c r="L5" s="15"/>
+      <c r="M5" s="15"/>
+      <c r="N5" s="15"/>
+    </row>
+    <row r="6" spans="1:18" ht="27.95" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A6" s="19"/>
+      <c r="B6" s="16"/>
+      <c r="C6" s="16"/>
+      <c r="D6" s="16"/>
+      <c r="E6" s="16"/>
+      <c r="F6" s="16"/>
+      <c r="G6" s="16"/>
+      <c r="H6" s="16"/>
+      <c r="I6" s="16"/>
+      <c r="J6" s="16"/>
+      <c r="K6" s="16"/>
+      <c r="L6" s="16"/>
+      <c r="M6" s="16"/>
+      <c r="N6" s="16"/>
+    </row>
+    <row r="7" spans="1:18" ht="27.95" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A7" s="17"/>
       <c r="B7" s="7"/>
       <c r="C7" s="7"/>
       <c r="D7" s="7"/>
@@ -15780,12 +16464,12 @@
       <c r="N7" s="7"/>
     </row>
     <row r="8" spans="1:18" ht="27.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A8" s="21"/>
+      <c r="A8" s="18"/>
       <c r="B8" s="15"/>
       <c r="C8" s="15"/>
       <c r="D8" s="15"/>
       <c r="E8" s="15"/>
-      <c r="F8" s="23"/>
+      <c r="F8" s="20"/>
       <c r="G8" s="15"/>
       <c r="H8" s="15"/>
       <c r="I8" s="15"/>
@@ -15796,12 +16480,12 @@
       <c r="N8" s="15"/>
     </row>
     <row r="9" spans="1:18" ht="27.95" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A9" s="22"/>
+      <c r="A9" s="19"/>
       <c r="B9" s="16"/>
       <c r="C9" s="16"/>
       <c r="D9" s="16"/>
       <c r="E9" s="16"/>
-      <c r="F9" s="24"/>
+      <c r="F9" s="21"/>
       <c r="G9" s="16"/>
       <c r="H9" s="16"/>
       <c r="I9" s="16"/>
@@ -15813,7 +16497,7 @@
       <c r="R9" s="10"/>
     </row>
     <row r="10" spans="1:18" ht="27.95" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A10" s="20"/>
+      <c r="A10" s="17"/>
       <c r="B10" s="7"/>
       <c r="C10" s="7"/>
       <c r="D10" s="7"/>
@@ -15829,7 +16513,7 @@
       <c r="N10" s="7"/>
     </row>
     <row r="11" spans="1:18" ht="27.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A11" s="21"/>
+      <c r="A11" s="18"/>
       <c r="B11" s="15"/>
       <c r="C11" s="15"/>
       <c r="D11" s="15"/>
@@ -15845,7 +16529,7 @@
       <c r="N11" s="15"/>
     </row>
     <row r="12" spans="1:18" ht="27.95" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A12" s="22"/>
+      <c r="A12" s="19"/>
       <c r="B12" s="16"/>
       <c r="C12" s="16"/>
       <c r="D12" s="16"/>
@@ -15861,7 +16545,7 @@
       <c r="N12" s="16"/>
     </row>
     <row r="13" spans="1:18" ht="27.95" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A13" s="20"/>
+      <c r="A13" s="17"/>
       <c r="B13" s="7"/>
       <c r="C13" s="7"/>
       <c r="D13" s="9"/>
@@ -15877,7 +16561,7 @@
       <c r="N13" s="7"/>
     </row>
     <row r="14" spans="1:18" ht="27.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A14" s="21"/>
+      <c r="A14" s="18"/>
       <c r="B14" s="15"/>
       <c r="C14" s="15"/>
       <c r="D14" s="15"/>
@@ -15893,7 +16577,7 @@
       <c r="N14" s="15"/>
     </row>
     <row r="15" spans="1:18" ht="27.95" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A15" s="22"/>
+      <c r="A15" s="19"/>
       <c r="B15" s="16"/>
       <c r="C15" s="16"/>
       <c r="D15" s="16"/>
@@ -15982,690 +16666,6 @@
     <mergeCell ref="L14:L15"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <drawing r:id="rId1"/>
-  <legacyDrawing r:id="rId2"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A9F6337B-89AA-4305-B4A8-6D5D44FBF989}">
-  <dimension ref="A1:R15"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="27.95" customHeight="1" x14ac:dyDescent="0.25"/>
-  <cols>
-    <col min="1" max="16384" width="11.42578125" style="6"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:18" ht="27.95" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="17"/>
-      <c r="B1" s="14" t="s">
-        <v>103</v>
-      </c>
-      <c r="C1" s="7" t="s">
-        <v>122</v>
-      </c>
-      <c r="D1" s="7"/>
-      <c r="E1" s="7"/>
-      <c r="F1" s="7"/>
-      <c r="G1" s="7"/>
-      <c r="H1" s="7"/>
-      <c r="I1" s="7"/>
-      <c r="J1" s="7"/>
-      <c r="K1" s="7"/>
-      <c r="L1" s="7"/>
-      <c r="M1" s="7"/>
-      <c r="N1" s="7"/>
-    </row>
-    <row r="2" spans="1:18" ht="27.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="18"/>
-      <c r="B2" s="15"/>
-      <c r="C2" s="15"/>
-      <c r="D2" s="15"/>
-      <c r="E2" s="15"/>
-      <c r="F2" s="15"/>
-      <c r="G2" s="15"/>
-      <c r="H2" s="15"/>
-      <c r="I2" s="15"/>
-      <c r="J2" s="15"/>
-      <c r="K2" s="15"/>
-      <c r="L2" s="15"/>
-      <c r="M2" s="15"/>
-      <c r="N2" s="15"/>
-    </row>
-    <row r="3" spans="1:18" ht="27.95" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="19"/>
-      <c r="B3" s="16"/>
-      <c r="C3" s="16"/>
-      <c r="D3" s="16"/>
-      <c r="E3" s="16"/>
-      <c r="F3" s="16"/>
-      <c r="G3" s="16"/>
-      <c r="H3" s="16"/>
-      <c r="I3" s="16"/>
-      <c r="J3" s="16"/>
-      <c r="K3" s="16"/>
-      <c r="L3" s="16"/>
-      <c r="M3" s="16"/>
-      <c r="N3" s="16"/>
-    </row>
-    <row r="4" spans="1:18" ht="27.95" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A4" s="20"/>
-      <c r="B4" s="14" t="s">
-        <v>104</v>
-      </c>
-      <c r="C4" s="7" t="s">
-        <v>109</v>
-      </c>
-      <c r="D4" s="7"/>
-      <c r="E4" s="7"/>
-      <c r="F4" s="7"/>
-      <c r="G4" s="7"/>
-      <c r="H4" s="7"/>
-      <c r="I4" s="7"/>
-      <c r="J4" s="7"/>
-      <c r="K4" s="7"/>
-      <c r="L4" s="7"/>
-      <c r="M4" s="7"/>
-      <c r="N4" s="7"/>
-    </row>
-    <row r="5" spans="1:18" ht="27.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="21"/>
-      <c r="B5" s="15"/>
-      <c r="C5" s="15"/>
-      <c r="D5" s="15"/>
-      <c r="E5" s="15"/>
-      <c r="F5" s="15"/>
-      <c r="G5" s="15"/>
-      <c r="H5" s="15"/>
-      <c r="I5" s="15"/>
-      <c r="J5" s="15"/>
-      <c r="K5" s="15"/>
-      <c r="L5" s="15"/>
-      <c r="M5" s="15"/>
-      <c r="N5" s="15"/>
-    </row>
-    <row r="6" spans="1:18" ht="27.95" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A6" s="22"/>
-      <c r="B6" s="16"/>
-      <c r="C6" s="16"/>
-      <c r="D6" s="16"/>
-      <c r="E6" s="16"/>
-      <c r="F6" s="16"/>
-      <c r="G6" s="16"/>
-      <c r="H6" s="16"/>
-      <c r="I6" s="16"/>
-      <c r="J6" s="16"/>
-      <c r="K6" s="16"/>
-      <c r="L6" s="16"/>
-      <c r="M6" s="16"/>
-      <c r="N6" s="16"/>
-    </row>
-    <row r="7" spans="1:18" ht="27.95" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A7" s="20" t="s">
-        <v>111</v>
-      </c>
-      <c r="B7" s="7" t="s">
-        <v>105</v>
-      </c>
-      <c r="C7" s="7" t="s">
-        <v>106</v>
-      </c>
-      <c r="D7" s="7" t="s">
-        <v>108</v>
-      </c>
-      <c r="E7" s="7" t="s">
-        <v>110</v>
-      </c>
-      <c r="F7" s="7" t="s">
-        <v>121</v>
-      </c>
-      <c r="G7" s="7"/>
-      <c r="H7" s="7"/>
-      <c r="I7" s="7"/>
-      <c r="J7" s="7"/>
-      <c r="K7" s="7"/>
-      <c r="L7" s="7"/>
-      <c r="M7" s="7"/>
-      <c r="N7" s="7"/>
-    </row>
-    <row r="8" spans="1:18" ht="27.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A8" s="21"/>
-      <c r="B8" s="15"/>
-      <c r="C8" s="15"/>
-      <c r="D8" s="15"/>
-      <c r="E8" s="15"/>
-      <c r="F8" s="15"/>
-      <c r="G8" s="15"/>
-      <c r="H8" s="15"/>
-      <c r="I8" s="15"/>
-      <c r="J8" s="15"/>
-      <c r="K8" s="15"/>
-      <c r="L8" s="15"/>
-      <c r="M8" s="15"/>
-      <c r="N8" s="15"/>
-    </row>
-    <row r="9" spans="1:18" ht="27.95" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A9" s="22"/>
-      <c r="B9" s="16"/>
-      <c r="C9" s="16"/>
-      <c r="D9" s="16"/>
-      <c r="E9" s="16"/>
-      <c r="F9" s="16"/>
-      <c r="G9" s="16"/>
-      <c r="H9" s="16"/>
-      <c r="I9" s="16"/>
-      <c r="J9" s="16"/>
-      <c r="K9" s="16"/>
-      <c r="L9" s="16"/>
-      <c r="M9" s="16"/>
-      <c r="N9" s="16"/>
-      <c r="R9" s="10"/>
-    </row>
-    <row r="10" spans="1:18" ht="27.95" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A10" s="20"/>
-      <c r="B10" s="7" t="s">
-        <v>107</v>
-      </c>
-      <c r="C10" s="7" t="s">
-        <v>112</v>
-      </c>
-      <c r="D10" s="7" t="s">
-        <v>113</v>
-      </c>
-      <c r="E10" s="7" t="s">
-        <v>114</v>
-      </c>
-      <c r="F10" s="7"/>
-      <c r="G10" s="7"/>
-      <c r="H10" s="7"/>
-      <c r="I10" s="7"/>
-      <c r="J10" s="7"/>
-      <c r="K10" s="7"/>
-      <c r="L10" s="7"/>
-      <c r="M10" s="7"/>
-      <c r="N10" s="7"/>
-    </row>
-    <row r="11" spans="1:18" ht="27.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A11" s="21"/>
-      <c r="B11" s="15"/>
-      <c r="C11" s="15"/>
-      <c r="D11" s="15"/>
-      <c r="E11" s="15"/>
-      <c r="F11" s="15"/>
-      <c r="G11" s="15"/>
-      <c r="H11" s="15"/>
-      <c r="I11" s="15"/>
-      <c r="J11" s="15"/>
-      <c r="K11" s="15"/>
-      <c r="L11" s="15"/>
-      <c r="M11" s="15"/>
-      <c r="N11" s="15"/>
-    </row>
-    <row r="12" spans="1:18" ht="27.95" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A12" s="22"/>
-      <c r="B12" s="16"/>
-      <c r="C12" s="16"/>
-      <c r="D12" s="16"/>
-      <c r="E12" s="16"/>
-      <c r="F12" s="16"/>
-      <c r="G12" s="16"/>
-      <c r="H12" s="16"/>
-      <c r="I12" s="16"/>
-      <c r="J12" s="16"/>
-      <c r="K12" s="16"/>
-      <c r="L12" s="16"/>
-      <c r="M12" s="16"/>
-      <c r="N12" s="16"/>
-    </row>
-    <row r="13" spans="1:18" ht="27.95" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A13" s="20"/>
-      <c r="B13" s="7"/>
-      <c r="C13" s="7"/>
-      <c r="D13" s="9"/>
-      <c r="E13" s="7"/>
-      <c r="F13" s="7"/>
-      <c r="G13" s="7"/>
-      <c r="H13" s="7"/>
-      <c r="I13" s="7"/>
-      <c r="J13" s="7"/>
-      <c r="K13" s="7"/>
-      <c r="L13" s="9"/>
-      <c r="M13" s="7"/>
-      <c r="N13" s="7"/>
-    </row>
-    <row r="14" spans="1:18" ht="27.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A14" s="21"/>
-      <c r="B14" s="15"/>
-      <c r="C14" s="15"/>
-      <c r="D14" s="15"/>
-      <c r="E14" s="15"/>
-      <c r="F14" s="15"/>
-      <c r="G14" s="15"/>
-      <c r="H14" s="15"/>
-      <c r="I14" s="15"/>
-      <c r="J14" s="15"/>
-      <c r="K14" s="15"/>
-      <c r="L14" s="15"/>
-      <c r="M14" s="15"/>
-      <c r="N14" s="15"/>
-    </row>
-    <row r="15" spans="1:18" ht="27.95" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A15" s="22"/>
-      <c r="B15" s="16"/>
-      <c r="C15" s="16"/>
-      <c r="D15" s="16"/>
-      <c r="E15" s="16"/>
-      <c r="F15" s="16"/>
-      <c r="G15" s="16"/>
-      <c r="H15" s="16"/>
-      <c r="I15" s="16"/>
-      <c r="J15" s="16"/>
-      <c r="K15" s="16"/>
-      <c r="L15" s="16"/>
-      <c r="M15" s="16"/>
-      <c r="N15" s="16"/>
-    </row>
-  </sheetData>
-  <mergeCells count="70">
-    <mergeCell ref="L2:L3"/>
-    <mergeCell ref="A1:A3"/>
-    <mergeCell ref="B2:B3"/>
-    <mergeCell ref="C2:C3"/>
-    <mergeCell ref="D2:D3"/>
-    <mergeCell ref="E2:E3"/>
-    <mergeCell ref="F2:F3"/>
-    <mergeCell ref="N5:N6"/>
-    <mergeCell ref="M2:M3"/>
-    <mergeCell ref="N2:N3"/>
-    <mergeCell ref="A4:A6"/>
-    <mergeCell ref="B5:B6"/>
-    <mergeCell ref="C5:C6"/>
-    <mergeCell ref="D5:D6"/>
-    <mergeCell ref="E5:E6"/>
-    <mergeCell ref="F5:F6"/>
-    <mergeCell ref="G5:G6"/>
-    <mergeCell ref="H5:H6"/>
-    <mergeCell ref="G2:G3"/>
-    <mergeCell ref="H2:H3"/>
-    <mergeCell ref="I2:I3"/>
-    <mergeCell ref="J2:J3"/>
-    <mergeCell ref="K2:K3"/>
-    <mergeCell ref="I5:I6"/>
-    <mergeCell ref="J5:J6"/>
-    <mergeCell ref="K5:K6"/>
-    <mergeCell ref="L5:L6"/>
-    <mergeCell ref="M5:M6"/>
-    <mergeCell ref="K8:K9"/>
-    <mergeCell ref="L8:L9"/>
-    <mergeCell ref="A7:A9"/>
-    <mergeCell ref="B8:B9"/>
-    <mergeCell ref="C8:C9"/>
-    <mergeCell ref="D8:D9"/>
-    <mergeCell ref="E8:E9"/>
-    <mergeCell ref="F8:F9"/>
-    <mergeCell ref="M11:M12"/>
-    <mergeCell ref="N11:N12"/>
-    <mergeCell ref="M8:M9"/>
-    <mergeCell ref="N8:N9"/>
-    <mergeCell ref="A10:A12"/>
-    <mergeCell ref="B11:B12"/>
-    <mergeCell ref="C11:C12"/>
-    <mergeCell ref="D11:D12"/>
-    <mergeCell ref="E11:E12"/>
-    <mergeCell ref="F11:F12"/>
-    <mergeCell ref="G11:G12"/>
-    <mergeCell ref="H11:H12"/>
-    <mergeCell ref="G8:G9"/>
-    <mergeCell ref="H8:H9"/>
-    <mergeCell ref="I8:I9"/>
-    <mergeCell ref="J8:J9"/>
-    <mergeCell ref="F14:F15"/>
-    <mergeCell ref="I11:I12"/>
-    <mergeCell ref="J11:J12"/>
-    <mergeCell ref="K11:K12"/>
-    <mergeCell ref="L11:L12"/>
-    <mergeCell ref="A13:A15"/>
-    <mergeCell ref="B14:B15"/>
-    <mergeCell ref="C14:C15"/>
-    <mergeCell ref="D14:D15"/>
-    <mergeCell ref="E14:E15"/>
-    <mergeCell ref="M14:M15"/>
-    <mergeCell ref="N14:N15"/>
-    <mergeCell ref="G14:G15"/>
-    <mergeCell ref="H14:H15"/>
-    <mergeCell ref="I14:I15"/>
-    <mergeCell ref="J14:J15"/>
-    <mergeCell ref="K14:K15"/>
-    <mergeCell ref="L14:L15"/>
-  </mergeCells>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <drawing r:id="rId1"/>
-  <legacyDrawing r:id="rId2"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{258ECD2D-C047-4967-AAA4-94D91ED5B3F1}">
-  <dimension ref="A1:R15"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="27.95" customHeight="1" x14ac:dyDescent="0.25"/>
-  <cols>
-    <col min="1" max="16384" width="11.42578125" style="6"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:18" ht="27.95" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="17"/>
-      <c r="B1" s="7"/>
-      <c r="C1" s="7"/>
-      <c r="D1" s="7"/>
-      <c r="E1" s="7"/>
-      <c r="F1" s="7"/>
-      <c r="G1" s="7"/>
-      <c r="H1" s="7"/>
-      <c r="I1" s="7"/>
-      <c r="J1" s="7"/>
-      <c r="K1" s="7"/>
-      <c r="L1" s="7"/>
-      <c r="M1" s="7"/>
-      <c r="N1" s="7"/>
-    </row>
-    <row r="2" spans="1:18" ht="27.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="18"/>
-      <c r="B2" s="15"/>
-      <c r="C2" s="15"/>
-      <c r="D2" s="15"/>
-      <c r="E2" s="15"/>
-      <c r="F2" s="15"/>
-      <c r="G2" s="15"/>
-      <c r="H2" s="15"/>
-      <c r="I2" s="15"/>
-      <c r="J2" s="15"/>
-      <c r="K2" s="15"/>
-      <c r="L2" s="15"/>
-      <c r="M2" s="15"/>
-      <c r="N2" s="15"/>
-    </row>
-    <row r="3" spans="1:18" ht="27.95" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="19"/>
-      <c r="B3" s="16"/>
-      <c r="C3" s="16"/>
-      <c r="D3" s="16"/>
-      <c r="E3" s="16"/>
-      <c r="F3" s="16"/>
-      <c r="G3" s="16"/>
-      <c r="H3" s="16"/>
-      <c r="I3" s="16"/>
-      <c r="J3" s="16"/>
-      <c r="K3" s="16"/>
-      <c r="L3" s="16"/>
-      <c r="M3" s="16"/>
-      <c r="N3" s="16"/>
-    </row>
-    <row r="4" spans="1:18" ht="27.95" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A4" s="20"/>
-      <c r="B4" s="7"/>
-      <c r="C4" s="7"/>
-      <c r="D4" s="7"/>
-      <c r="E4" s="7"/>
-      <c r="F4" s="7"/>
-      <c r="G4" s="7"/>
-      <c r="H4" s="7"/>
-      <c r="I4" s="7"/>
-      <c r="J4" s="7"/>
-      <c r="K4" s="7"/>
-      <c r="L4" s="7"/>
-      <c r="M4" s="7"/>
-      <c r="N4" s="7"/>
-    </row>
-    <row r="5" spans="1:18" ht="27.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="21"/>
-      <c r="B5" s="15"/>
-      <c r="C5" s="15"/>
-      <c r="D5" s="15"/>
-      <c r="E5" s="15"/>
-      <c r="F5" s="15"/>
-      <c r="G5" s="15"/>
-      <c r="H5" s="15"/>
-      <c r="I5" s="15"/>
-      <c r="J5" s="15"/>
-      <c r="K5" s="15"/>
-      <c r="L5" s="15"/>
-      <c r="M5" s="15"/>
-      <c r="N5" s="15"/>
-    </row>
-    <row r="6" spans="1:18" ht="27.95" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A6" s="22"/>
-      <c r="B6" s="16"/>
-      <c r="C6" s="16"/>
-      <c r="D6" s="16"/>
-      <c r="E6" s="16"/>
-      <c r="F6" s="16"/>
-      <c r="G6" s="16"/>
-      <c r="H6" s="16"/>
-      <c r="I6" s="16"/>
-      <c r="J6" s="16"/>
-      <c r="K6" s="16"/>
-      <c r="L6" s="16"/>
-      <c r="M6" s="16"/>
-      <c r="N6" s="16"/>
-    </row>
-    <row r="7" spans="1:18" ht="27.95" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A7" s="20"/>
-      <c r="B7" s="7"/>
-      <c r="C7" s="7"/>
-      <c r="D7" s="7"/>
-      <c r="E7" s="7"/>
-      <c r="F7" s="9"/>
-      <c r="G7" s="7"/>
-      <c r="H7" s="7"/>
-      <c r="I7" s="7"/>
-      <c r="J7" s="7"/>
-      <c r="K7" s="7"/>
-      <c r="L7" s="7"/>
-      <c r="M7" s="7"/>
-      <c r="N7" s="7"/>
-    </row>
-    <row r="8" spans="1:18" ht="27.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A8" s="21"/>
-      <c r="B8" s="15"/>
-      <c r="C8" s="15"/>
-      <c r="D8" s="15"/>
-      <c r="E8" s="15"/>
-      <c r="F8" s="23"/>
-      <c r="G8" s="15"/>
-      <c r="H8" s="15"/>
-      <c r="I8" s="15"/>
-      <c r="J8" s="15"/>
-      <c r="K8" s="15"/>
-      <c r="L8" s="15"/>
-      <c r="M8" s="15"/>
-      <c r="N8" s="15"/>
-    </row>
-    <row r="9" spans="1:18" ht="27.95" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A9" s="22"/>
-      <c r="B9" s="16"/>
-      <c r="C9" s="16"/>
-      <c r="D9" s="16"/>
-      <c r="E9" s="16"/>
-      <c r="F9" s="24"/>
-      <c r="G9" s="16"/>
-      <c r="H9" s="16"/>
-      <c r="I9" s="16"/>
-      <c r="J9" s="16"/>
-      <c r="K9" s="16"/>
-      <c r="L9" s="16"/>
-      <c r="M9" s="16"/>
-      <c r="N9" s="16"/>
-      <c r="R9" s="10"/>
-    </row>
-    <row r="10" spans="1:18" ht="27.95" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A10" s="20"/>
-      <c r="B10" s="7"/>
-      <c r="C10" s="7"/>
-      <c r="D10" s="7"/>
-      <c r="E10" s="8"/>
-      <c r="F10" s="7"/>
-      <c r="G10" s="7"/>
-      <c r="H10" s="7"/>
-      <c r="I10" s="7"/>
-      <c r="J10" s="7"/>
-      <c r="K10" s="7"/>
-      <c r="L10" s="7"/>
-      <c r="M10" s="7"/>
-      <c r="N10" s="7"/>
-    </row>
-    <row r="11" spans="1:18" ht="27.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A11" s="21"/>
-      <c r="B11" s="15"/>
-      <c r="C11" s="15"/>
-      <c r="D11" s="15"/>
-      <c r="E11" s="15"/>
-      <c r="F11" s="15"/>
-      <c r="G11" s="15"/>
-      <c r="H11" s="15"/>
-      <c r="I11" s="15"/>
-      <c r="J11" s="15"/>
-      <c r="K11" s="15"/>
-      <c r="L11" s="15"/>
-      <c r="M11" s="15"/>
-      <c r="N11" s="15"/>
-    </row>
-    <row r="12" spans="1:18" ht="27.95" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A12" s="22"/>
-      <c r="B12" s="16"/>
-      <c r="C12" s="16"/>
-      <c r="D12" s="16"/>
-      <c r="E12" s="16"/>
-      <c r="F12" s="16"/>
-      <c r="G12" s="16"/>
-      <c r="H12" s="16"/>
-      <c r="I12" s="16"/>
-      <c r="J12" s="16"/>
-      <c r="K12" s="16"/>
-      <c r="L12" s="16"/>
-      <c r="M12" s="16"/>
-      <c r="N12" s="16"/>
-    </row>
-    <row r="13" spans="1:18" ht="27.95" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A13" s="20"/>
-      <c r="B13" s="7"/>
-      <c r="C13" s="7"/>
-      <c r="D13" s="9"/>
-      <c r="E13" s="7"/>
-      <c r="F13" s="7"/>
-      <c r="G13" s="7"/>
-      <c r="H13" s="7"/>
-      <c r="I13" s="7"/>
-      <c r="J13" s="7"/>
-      <c r="K13" s="7"/>
-      <c r="L13" s="9"/>
-      <c r="M13" s="7"/>
-      <c r="N13" s="7"/>
-    </row>
-    <row r="14" spans="1:18" ht="27.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A14" s="21"/>
-      <c r="B14" s="15"/>
-      <c r="C14" s="15"/>
-      <c r="D14" s="15"/>
-      <c r="E14" s="15"/>
-      <c r="F14" s="15"/>
-      <c r="G14" s="15"/>
-      <c r="H14" s="15"/>
-      <c r="I14" s="15"/>
-      <c r="J14" s="15"/>
-      <c r="K14" s="15"/>
-      <c r="L14" s="15"/>
-      <c r="M14" s="15"/>
-      <c r="N14" s="15"/>
-    </row>
-    <row r="15" spans="1:18" ht="27.95" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A15" s="22"/>
-      <c r="B15" s="16"/>
-      <c r="C15" s="16"/>
-      <c r="D15" s="16"/>
-      <c r="E15" s="16"/>
-      <c r="F15" s="16"/>
-      <c r="G15" s="16"/>
-      <c r="H15" s="16"/>
-      <c r="I15" s="16"/>
-      <c r="J15" s="16"/>
-      <c r="K15" s="16"/>
-      <c r="L15" s="16"/>
-      <c r="M15" s="16"/>
-      <c r="N15" s="16"/>
-    </row>
-  </sheetData>
-  <mergeCells count="70">
-    <mergeCell ref="M14:M15"/>
-    <mergeCell ref="N14:N15"/>
-    <mergeCell ref="G14:G15"/>
-    <mergeCell ref="H14:H15"/>
-    <mergeCell ref="I14:I15"/>
-    <mergeCell ref="J14:J15"/>
-    <mergeCell ref="K14:K15"/>
-    <mergeCell ref="L14:L15"/>
-    <mergeCell ref="A13:A15"/>
-    <mergeCell ref="B14:B15"/>
-    <mergeCell ref="C14:C15"/>
-    <mergeCell ref="D14:D15"/>
-    <mergeCell ref="E14:E15"/>
-    <mergeCell ref="F14:F15"/>
-    <mergeCell ref="I11:I12"/>
-    <mergeCell ref="J11:J12"/>
-    <mergeCell ref="K11:K12"/>
-    <mergeCell ref="L11:L12"/>
-    <mergeCell ref="M11:M12"/>
-    <mergeCell ref="N11:N12"/>
-    <mergeCell ref="M8:M9"/>
-    <mergeCell ref="N8:N9"/>
-    <mergeCell ref="A10:A12"/>
-    <mergeCell ref="B11:B12"/>
-    <mergeCell ref="C11:C12"/>
-    <mergeCell ref="D11:D12"/>
-    <mergeCell ref="E11:E12"/>
-    <mergeCell ref="F11:F12"/>
-    <mergeCell ref="G11:G12"/>
-    <mergeCell ref="H11:H12"/>
-    <mergeCell ref="G8:G9"/>
-    <mergeCell ref="H8:H9"/>
-    <mergeCell ref="I8:I9"/>
-    <mergeCell ref="J8:J9"/>
-    <mergeCell ref="K8:K9"/>
-    <mergeCell ref="L8:L9"/>
-    <mergeCell ref="A7:A9"/>
-    <mergeCell ref="B8:B9"/>
-    <mergeCell ref="C8:C9"/>
-    <mergeCell ref="D8:D9"/>
-    <mergeCell ref="E8:E9"/>
-    <mergeCell ref="F8:F9"/>
-    <mergeCell ref="I5:I6"/>
-    <mergeCell ref="J5:J6"/>
-    <mergeCell ref="K5:K6"/>
-    <mergeCell ref="L5:L6"/>
-    <mergeCell ref="M5:M6"/>
-    <mergeCell ref="N5:N6"/>
-    <mergeCell ref="M2:M3"/>
-    <mergeCell ref="N2:N3"/>
-    <mergeCell ref="A4:A6"/>
-    <mergeCell ref="B5:B6"/>
-    <mergeCell ref="C5:C6"/>
-    <mergeCell ref="D5:D6"/>
-    <mergeCell ref="E5:E6"/>
-    <mergeCell ref="F5:F6"/>
-    <mergeCell ref="G5:G6"/>
-    <mergeCell ref="H5:H6"/>
-    <mergeCell ref="G2:G3"/>
-    <mergeCell ref="H2:H3"/>
-    <mergeCell ref="I2:I3"/>
-    <mergeCell ref="J2:J3"/>
-    <mergeCell ref="K2:K3"/>
-    <mergeCell ref="L2:L3"/>
-    <mergeCell ref="A1:A3"/>
-    <mergeCell ref="B2:B3"/>
-    <mergeCell ref="C2:C3"/>
-    <mergeCell ref="D2:D3"/>
-    <mergeCell ref="E2:E3"/>
-    <mergeCell ref="F2:F3"/>
-  </mergeCells>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <legacyDrawing r:id="rId1"/>
 </worksheet>
 </file>
@@ -16679,7 +16679,7 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:18" ht="27.95" customHeight="1" thickBot="1" x14ac:dyDescent="0.6">
-      <c r="A1" s="17" t="s">
+      <c r="A1" s="22" t="s">
         <v>0</v>
       </c>
       <c r="B1" s="11" t="s">
@@ -16718,7 +16718,7 @@
       <c r="Q1" s="7"/>
     </row>
     <row r="2" spans="1:18" ht="27.95" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A2" s="18"/>
+      <c r="A2" s="23"/>
       <c r="B2" s="15"/>
       <c r="C2" s="15"/>
       <c r="D2" s="15"/>
@@ -16737,7 +16737,7 @@
       <c r="Q2" s="15"/>
     </row>
     <row r="3" spans="1:18" ht="27.95" customHeight="1" thickBot="1" x14ac:dyDescent="0.6">
-      <c r="A3" s="19"/>
+      <c r="A3" s="24"/>
       <c r="B3" s="16"/>
       <c r="C3" s="16"/>
       <c r="D3" s="16"/>
@@ -16756,7 +16756,7 @@
       <c r="Q3" s="16"/>
     </row>
     <row r="4" spans="1:18" ht="27.95" customHeight="1" thickBot="1" x14ac:dyDescent="0.6">
-      <c r="A4" s="20" t="s">
+      <c r="A4" s="17" t="s">
         <v>2</v>
       </c>
       <c r="B4" s="7" t="s">
@@ -16803,7 +16803,7 @@
       <c r="Q4" s="7"/>
     </row>
     <row r="5" spans="1:18" ht="27.95" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A5" s="21"/>
+      <c r="A5" s="18"/>
       <c r="B5" s="15"/>
       <c r="C5" s="15"/>
       <c r="D5" s="15"/>
@@ -16822,7 +16822,7 @@
       <c r="Q5" s="15"/>
     </row>
     <row r="6" spans="1:18" ht="27.95" customHeight="1" thickBot="1" x14ac:dyDescent="0.6">
-      <c r="A6" s="22"/>
+      <c r="A6" s="19"/>
       <c r="B6" s="16"/>
       <c r="C6" s="16"/>
       <c r="D6" s="16"/>
@@ -16841,7 +16841,7 @@
       <c r="Q6" s="16"/>
     </row>
     <row r="7" spans="1:18" ht="27.95" customHeight="1" thickBot="1" x14ac:dyDescent="0.6">
-      <c r="A7" s="20" t="s">
+      <c r="A7" s="17" t="s">
         <v>1</v>
       </c>
       <c r="B7" s="7" t="s">
@@ -16897,12 +16897,12 @@
       </c>
     </row>
     <row r="8" spans="1:18" ht="27.95" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A8" s="21"/>
+      <c r="A8" s="18"/>
       <c r="B8" s="15"/>
       <c r="C8" s="15"/>
       <c r="D8" s="15"/>
       <c r="E8" s="15"/>
-      <c r="F8" s="23"/>
+      <c r="F8" s="20"/>
       <c r="G8" s="15"/>
       <c r="H8" s="15"/>
       <c r="I8" s="15"/>
@@ -16917,12 +16917,12 @@
       <c r="R8" s="15"/>
     </row>
     <row r="9" spans="1:18" ht="27.95" customHeight="1" thickBot="1" x14ac:dyDescent="0.6">
-      <c r="A9" s="22"/>
+      <c r="A9" s="19"/>
       <c r="B9" s="16"/>
       <c r="C9" s="16"/>
       <c r="D9" s="16"/>
       <c r="E9" s="16"/>
-      <c r="F9" s="24"/>
+      <c r="F9" s="21"/>
       <c r="G9" s="16"/>
       <c r="H9" s="16"/>
       <c r="I9" s="16"/>
@@ -16937,7 +16937,7 @@
       <c r="R9" s="16"/>
     </row>
     <row r="10" spans="1:18" ht="27.95" customHeight="1" thickBot="1" x14ac:dyDescent="0.6">
-      <c r="A10" s="20" t="s">
+      <c r="A10" s="17" t="s">
         <v>3</v>
       </c>
       <c r="B10" s="7" t="s">
@@ -16972,7 +16972,7 @@
       <c r="Q10" s="7"/>
     </row>
     <row r="11" spans="1:18" ht="27.95" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A11" s="21"/>
+      <c r="A11" s="18"/>
       <c r="B11" s="15"/>
       <c r="C11" s="15"/>
       <c r="D11" s="15"/>
@@ -16991,7 +16991,7 @@
       <c r="Q11" s="15"/>
     </row>
     <row r="12" spans="1:18" ht="27.95" customHeight="1" thickBot="1" x14ac:dyDescent="0.6">
-      <c r="A12" s="22"/>
+      <c r="A12" s="19"/>
       <c r="B12" s="16"/>
       <c r="C12" s="16"/>
       <c r="D12" s="16"/>
@@ -17010,7 +17010,7 @@
       <c r="Q12" s="16"/>
     </row>
     <row r="13" spans="1:18" ht="27.95" customHeight="1" thickBot="1" x14ac:dyDescent="0.6">
-      <c r="A13" s="20" t="s">
+      <c r="A13" s="17" t="s">
         <v>59</v>
       </c>
       <c r="B13" s="13" t="s">
@@ -17041,7 +17041,7 @@
       <c r="Q13" s="7"/>
     </row>
     <row r="14" spans="1:18" ht="27.95" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A14" s="21"/>
+      <c r="A14" s="18"/>
       <c r="B14" s="15"/>
       <c r="C14" s="15"/>
       <c r="D14" s="15"/>
@@ -17060,7 +17060,7 @@
       <c r="Q14" s="15"/>
     </row>
     <row r="15" spans="1:18" ht="27.95" customHeight="1" thickBot="1" x14ac:dyDescent="0.6">
-      <c r="A15" s="22"/>
+      <c r="A15" s="19"/>
       <c r="B15" s="16"/>
       <c r="C15" s="16"/>
       <c r="D15" s="16"/>
@@ -18083,30 +18083,52 @@
     </row>
   </sheetData>
   <mergeCells count="86">
-    <mergeCell ref="Q11:Q12"/>
-    <mergeCell ref="Q14:Q15"/>
-    <mergeCell ref="R8:R9"/>
-    <mergeCell ref="Q8:Q9"/>
-    <mergeCell ref="P8:P9"/>
-    <mergeCell ref="O2:O3"/>
-    <mergeCell ref="O5:O6"/>
-    <mergeCell ref="O8:O9"/>
-    <mergeCell ref="P2:P3"/>
-    <mergeCell ref="Q2:Q3"/>
-    <mergeCell ref="Q5:Q6"/>
-    <mergeCell ref="O11:O12"/>
-    <mergeCell ref="P5:P6"/>
-    <mergeCell ref="P11:P12"/>
-    <mergeCell ref="O14:O15"/>
-    <mergeCell ref="L14:L15"/>
-    <mergeCell ref="M14:M15"/>
-    <mergeCell ref="N14:N15"/>
-    <mergeCell ref="M11:M12"/>
-    <mergeCell ref="N11:N12"/>
-    <mergeCell ref="M5:M6"/>
-    <mergeCell ref="N5:N6"/>
-    <mergeCell ref="P14:P15"/>
-    <mergeCell ref="N8:N9"/>
+    <mergeCell ref="L2:L3"/>
+    <mergeCell ref="L5:L6"/>
+    <mergeCell ref="L8:L9"/>
+    <mergeCell ref="L11:L12"/>
+    <mergeCell ref="M8:M9"/>
+    <mergeCell ref="M2:M3"/>
+    <mergeCell ref="J2:J3"/>
+    <mergeCell ref="J5:J6"/>
+    <mergeCell ref="J8:J9"/>
+    <mergeCell ref="J11:J12"/>
+    <mergeCell ref="K2:K3"/>
+    <mergeCell ref="K5:K6"/>
+    <mergeCell ref="K8:K9"/>
+    <mergeCell ref="K11:K12"/>
+    <mergeCell ref="E2:E3"/>
+    <mergeCell ref="B8:B9"/>
+    <mergeCell ref="C2:C3"/>
+    <mergeCell ref="C5:C6"/>
+    <mergeCell ref="D2:D3"/>
+    <mergeCell ref="D5:D6"/>
+    <mergeCell ref="E5:E6"/>
+    <mergeCell ref="A1:A3"/>
+    <mergeCell ref="A4:A6"/>
+    <mergeCell ref="A7:A9"/>
+    <mergeCell ref="A10:A12"/>
+    <mergeCell ref="C8:C9"/>
+    <mergeCell ref="B2:B3"/>
+    <mergeCell ref="B11:B12"/>
+    <mergeCell ref="C11:C12"/>
+    <mergeCell ref="B5:B6"/>
+    <mergeCell ref="A13:A15"/>
+    <mergeCell ref="I2:I3"/>
+    <mergeCell ref="I5:I6"/>
+    <mergeCell ref="F11:F12"/>
+    <mergeCell ref="G11:G12"/>
+    <mergeCell ref="H11:H12"/>
+    <mergeCell ref="I11:I12"/>
+    <mergeCell ref="H8:H9"/>
+    <mergeCell ref="I8:I9"/>
+    <mergeCell ref="F2:F3"/>
+    <mergeCell ref="G2:G3"/>
+    <mergeCell ref="F8:F9"/>
+    <mergeCell ref="G8:G9"/>
+    <mergeCell ref="H2:H3"/>
+    <mergeCell ref="G5:G6"/>
+    <mergeCell ref="H5:H6"/>
     <mergeCell ref="N2:N3"/>
     <mergeCell ref="B14:B15"/>
     <mergeCell ref="C14:C15"/>
@@ -18123,52 +18145,30 @@
     <mergeCell ref="E8:E9"/>
     <mergeCell ref="D11:D12"/>
     <mergeCell ref="E11:E12"/>
-    <mergeCell ref="A13:A15"/>
-    <mergeCell ref="I2:I3"/>
-    <mergeCell ref="I5:I6"/>
-    <mergeCell ref="F11:F12"/>
-    <mergeCell ref="G11:G12"/>
-    <mergeCell ref="H11:H12"/>
-    <mergeCell ref="I11:I12"/>
-    <mergeCell ref="H8:H9"/>
-    <mergeCell ref="I8:I9"/>
-    <mergeCell ref="F2:F3"/>
-    <mergeCell ref="G2:G3"/>
-    <mergeCell ref="F8:F9"/>
-    <mergeCell ref="G8:G9"/>
-    <mergeCell ref="H2:H3"/>
-    <mergeCell ref="G5:G6"/>
-    <mergeCell ref="H5:H6"/>
-    <mergeCell ref="A1:A3"/>
-    <mergeCell ref="A4:A6"/>
-    <mergeCell ref="A7:A9"/>
-    <mergeCell ref="A10:A12"/>
-    <mergeCell ref="C8:C9"/>
-    <mergeCell ref="B2:B3"/>
-    <mergeCell ref="B11:B12"/>
-    <mergeCell ref="C11:C12"/>
-    <mergeCell ref="B5:B6"/>
-    <mergeCell ref="E2:E3"/>
-    <mergeCell ref="B8:B9"/>
-    <mergeCell ref="C2:C3"/>
-    <mergeCell ref="C5:C6"/>
-    <mergeCell ref="D2:D3"/>
-    <mergeCell ref="D5:D6"/>
-    <mergeCell ref="E5:E6"/>
-    <mergeCell ref="J2:J3"/>
-    <mergeCell ref="J5:J6"/>
-    <mergeCell ref="J8:J9"/>
-    <mergeCell ref="J11:J12"/>
-    <mergeCell ref="K2:K3"/>
-    <mergeCell ref="K5:K6"/>
-    <mergeCell ref="K8:K9"/>
-    <mergeCell ref="K11:K12"/>
-    <mergeCell ref="L2:L3"/>
-    <mergeCell ref="L5:L6"/>
-    <mergeCell ref="L8:L9"/>
-    <mergeCell ref="L11:L12"/>
-    <mergeCell ref="M8:M9"/>
-    <mergeCell ref="M2:M3"/>
+    <mergeCell ref="O11:O12"/>
+    <mergeCell ref="P5:P6"/>
+    <mergeCell ref="P11:P12"/>
+    <mergeCell ref="O14:O15"/>
+    <mergeCell ref="L14:L15"/>
+    <mergeCell ref="M14:M15"/>
+    <mergeCell ref="N14:N15"/>
+    <mergeCell ref="M11:M12"/>
+    <mergeCell ref="N11:N12"/>
+    <mergeCell ref="M5:M6"/>
+    <mergeCell ref="N5:N6"/>
+    <mergeCell ref="P14:P15"/>
+    <mergeCell ref="N8:N9"/>
+    <mergeCell ref="O2:O3"/>
+    <mergeCell ref="O5:O6"/>
+    <mergeCell ref="O8:O9"/>
+    <mergeCell ref="P2:P3"/>
+    <mergeCell ref="Q2:Q3"/>
+    <mergeCell ref="Q5:Q6"/>
+    <mergeCell ref="Q11:Q12"/>
+    <mergeCell ref="Q14:Q15"/>
+    <mergeCell ref="R8:R9"/>
+    <mergeCell ref="Q8:Q9"/>
+    <mergeCell ref="P8:P9"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -18185,7 +18185,7 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:18" ht="27.95" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="17" t="s">
+      <c r="A1" s="22" t="s">
         <v>4</v>
       </c>
       <c r="B1" s="7" t="s">
@@ -18225,7 +18225,7 @@
       <c r="N1" s="7"/>
     </row>
     <row r="2" spans="1:18" ht="27.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="18"/>
+      <c r="A2" s="23"/>
       <c r="B2" s="15"/>
       <c r="C2" s="15"/>
       <c r="D2" s="15"/>
@@ -18241,7 +18241,7 @@
       <c r="N2" s="15"/>
     </row>
     <row r="3" spans="1:18" ht="27.95" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="19"/>
+      <c r="A3" s="24"/>
       <c r="B3" s="16"/>
       <c r="C3" s="16"/>
       <c r="D3" s="16"/>
@@ -18257,7 +18257,7 @@
       <c r="N3" s="16"/>
     </row>
     <row r="4" spans="1:18" ht="27.95" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A4" s="20" t="s">
+      <c r="A4" s="17" t="s">
         <v>5</v>
       </c>
       <c r="B4" s="7" t="s">
@@ -18299,7 +18299,7 @@
       <c r="N4" s="7"/>
     </row>
     <row r="5" spans="1:18" ht="27.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="21"/>
+      <c r="A5" s="18"/>
       <c r="B5" s="15"/>
       <c r="C5" s="15"/>
       <c r="D5" s="15"/>
@@ -18315,7 +18315,7 @@
       <c r="N5" s="15"/>
     </row>
     <row r="6" spans="1:18" ht="27.95" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A6" s="22"/>
+      <c r="A6" s="19"/>
       <c r="B6" s="16"/>
       <c r="C6" s="16"/>
       <c r="D6" s="16"/>
@@ -18331,7 +18331,7 @@
       <c r="N6" s="16"/>
     </row>
     <row r="7" spans="1:18" ht="27.95" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A7" s="20" t="s">
+      <c r="A7" s="17" t="s">
         <v>6</v>
       </c>
       <c r="B7" s="7" t="s">
@@ -18359,12 +18359,12 @@
       <c r="N7" s="7"/>
     </row>
     <row r="8" spans="1:18" ht="27.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A8" s="21"/>
+      <c r="A8" s="18"/>
       <c r="B8" s="15"/>
       <c r="C8" s="15"/>
       <c r="D8" s="15"/>
       <c r="E8" s="15"/>
-      <c r="F8" s="23"/>
+      <c r="F8" s="20"/>
       <c r="G8" s="15"/>
       <c r="H8" s="15"/>
       <c r="I8" s="15"/>
@@ -18375,12 +18375,12 @@
       <c r="N8" s="15"/>
     </row>
     <row r="9" spans="1:18" ht="27.95" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A9" s="22"/>
+      <c r="A9" s="19"/>
       <c r="B9" s="16"/>
       <c r="C9" s="16"/>
       <c r="D9" s="16"/>
       <c r="E9" s="16"/>
-      <c r="F9" s="24"/>
+      <c r="F9" s="21"/>
       <c r="G9" s="16"/>
       <c r="H9" s="16"/>
       <c r="I9" s="16"/>
@@ -18392,7 +18392,7 @@
       <c r="R9" s="10"/>
     </row>
     <row r="10" spans="1:18" ht="27.95" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A10" s="20" t="s">
+      <c r="A10" s="17" t="s">
         <v>0</v>
       </c>
       <c r="B10" s="7" t="s">
@@ -18418,7 +18418,7 @@
       <c r="N10" s="7"/>
     </row>
     <row r="11" spans="1:18" ht="27.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A11" s="21"/>
+      <c r="A11" s="18"/>
       <c r="B11" s="15"/>
       <c r="C11" s="15"/>
       <c r="D11" s="15"/>
@@ -18434,7 +18434,7 @@
       <c r="N11" s="15"/>
     </row>
     <row r="12" spans="1:18" ht="27.95" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A12" s="22"/>
+      <c r="A12" s="19"/>
       <c r="B12" s="16"/>
       <c r="C12" s="16"/>
       <c r="D12" s="16"/>
@@ -18450,7 +18450,7 @@
       <c r="N12" s="16"/>
     </row>
     <row r="13" spans="1:18" ht="27.95" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A13" s="20" t="s">
+      <c r="A13" s="17" t="s">
         <v>7</v>
       </c>
       <c r="B13" s="7" t="s">
@@ -18494,7 +18494,7 @@
       </c>
     </row>
     <row r="14" spans="1:18" ht="27.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A14" s="21"/>
+      <c r="A14" s="18"/>
       <c r="B14" s="15"/>
       <c r="C14" s="15"/>
       <c r="D14" s="15"/>
@@ -18510,7 +18510,7 @@
       <c r="N14" s="15"/>
     </row>
     <row r="15" spans="1:18" ht="27.95" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A15" s="22"/>
+      <c r="A15" s="19"/>
       <c r="B15" s="16"/>
       <c r="C15" s="16"/>
       <c r="D15" s="16"/>
@@ -18527,64 +18527,6 @@
     </row>
   </sheetData>
   <mergeCells count="70">
-    <mergeCell ref="N14:N15"/>
-    <mergeCell ref="N2:N3"/>
-    <mergeCell ref="M5:M6"/>
-    <mergeCell ref="N5:N6"/>
-    <mergeCell ref="M11:M12"/>
-    <mergeCell ref="N11:N12"/>
-    <mergeCell ref="M2:M3"/>
-    <mergeCell ref="M8:M9"/>
-    <mergeCell ref="N8:N9"/>
-    <mergeCell ref="K8:K9"/>
-    <mergeCell ref="L8:L9"/>
-    <mergeCell ref="K5:K6"/>
-    <mergeCell ref="L5:L6"/>
-    <mergeCell ref="M14:M15"/>
-    <mergeCell ref="K11:K12"/>
-    <mergeCell ref="L11:L12"/>
-    <mergeCell ref="K14:K15"/>
-    <mergeCell ref="L14:L15"/>
-    <mergeCell ref="A13:A15"/>
-    <mergeCell ref="G14:G15"/>
-    <mergeCell ref="H14:H15"/>
-    <mergeCell ref="I14:I15"/>
-    <mergeCell ref="J14:J15"/>
-    <mergeCell ref="D14:D15"/>
-    <mergeCell ref="E14:E15"/>
-    <mergeCell ref="F14:F15"/>
-    <mergeCell ref="A10:A12"/>
-    <mergeCell ref="B11:B12"/>
-    <mergeCell ref="C11:C12"/>
-    <mergeCell ref="D11:D12"/>
-    <mergeCell ref="E11:E12"/>
-    <mergeCell ref="I11:I12"/>
-    <mergeCell ref="J11:J12"/>
-    <mergeCell ref="F11:F12"/>
-    <mergeCell ref="G11:G12"/>
-    <mergeCell ref="B14:B15"/>
-    <mergeCell ref="C14:C15"/>
-    <mergeCell ref="H11:H12"/>
-    <mergeCell ref="A7:A9"/>
-    <mergeCell ref="B8:B9"/>
-    <mergeCell ref="C8:C9"/>
-    <mergeCell ref="D8:D9"/>
-    <mergeCell ref="E8:E9"/>
-    <mergeCell ref="F8:F9"/>
-    <mergeCell ref="G5:G6"/>
-    <mergeCell ref="H5:H6"/>
-    <mergeCell ref="I5:I6"/>
-    <mergeCell ref="J5:J6"/>
-    <mergeCell ref="F5:F6"/>
-    <mergeCell ref="G8:G9"/>
-    <mergeCell ref="H8:H9"/>
-    <mergeCell ref="I8:I9"/>
-    <mergeCell ref="J8:J9"/>
-    <mergeCell ref="A4:A6"/>
-    <mergeCell ref="B5:B6"/>
-    <mergeCell ref="C5:C6"/>
-    <mergeCell ref="D5:D6"/>
-    <mergeCell ref="E5:E6"/>
     <mergeCell ref="L2:L3"/>
     <mergeCell ref="A1:A3"/>
     <mergeCell ref="B2:B3"/>
@@ -18597,6 +18539,64 @@
     <mergeCell ref="I2:I3"/>
     <mergeCell ref="J2:J3"/>
     <mergeCell ref="K2:K3"/>
+    <mergeCell ref="A4:A6"/>
+    <mergeCell ref="B5:B6"/>
+    <mergeCell ref="C5:C6"/>
+    <mergeCell ref="D5:D6"/>
+    <mergeCell ref="E5:E6"/>
+    <mergeCell ref="F8:F9"/>
+    <mergeCell ref="G5:G6"/>
+    <mergeCell ref="H5:H6"/>
+    <mergeCell ref="I5:I6"/>
+    <mergeCell ref="J5:J6"/>
+    <mergeCell ref="F5:F6"/>
+    <mergeCell ref="G8:G9"/>
+    <mergeCell ref="H8:H9"/>
+    <mergeCell ref="I8:I9"/>
+    <mergeCell ref="J8:J9"/>
+    <mergeCell ref="A7:A9"/>
+    <mergeCell ref="B8:B9"/>
+    <mergeCell ref="C8:C9"/>
+    <mergeCell ref="D8:D9"/>
+    <mergeCell ref="E8:E9"/>
+    <mergeCell ref="I11:I12"/>
+    <mergeCell ref="J11:J12"/>
+    <mergeCell ref="F11:F12"/>
+    <mergeCell ref="G11:G12"/>
+    <mergeCell ref="B14:B15"/>
+    <mergeCell ref="C14:C15"/>
+    <mergeCell ref="H11:H12"/>
+    <mergeCell ref="A10:A12"/>
+    <mergeCell ref="B11:B12"/>
+    <mergeCell ref="C11:C12"/>
+    <mergeCell ref="D11:D12"/>
+    <mergeCell ref="E11:E12"/>
+    <mergeCell ref="A13:A15"/>
+    <mergeCell ref="G14:G15"/>
+    <mergeCell ref="H14:H15"/>
+    <mergeCell ref="I14:I15"/>
+    <mergeCell ref="J14:J15"/>
+    <mergeCell ref="D14:D15"/>
+    <mergeCell ref="E14:E15"/>
+    <mergeCell ref="F14:F15"/>
+    <mergeCell ref="K8:K9"/>
+    <mergeCell ref="L8:L9"/>
+    <mergeCell ref="K5:K6"/>
+    <mergeCell ref="L5:L6"/>
+    <mergeCell ref="M14:M15"/>
+    <mergeCell ref="K11:K12"/>
+    <mergeCell ref="L11:L12"/>
+    <mergeCell ref="K14:K15"/>
+    <mergeCell ref="L14:L15"/>
+    <mergeCell ref="N14:N15"/>
+    <mergeCell ref="N2:N3"/>
+    <mergeCell ref="M5:M6"/>
+    <mergeCell ref="N5:N6"/>
+    <mergeCell ref="M11:M12"/>
+    <mergeCell ref="N11:N12"/>
+    <mergeCell ref="M2:M3"/>
+    <mergeCell ref="M8:M9"/>
+    <mergeCell ref="N8:N9"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>

</xml_diff>